<commit_message>
adicionando novos campos nas fatos e na dim
</commit_message>
<xml_diff>
--- a/new_issues.xlsx
+++ b/new_issues.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://bcpsec-my.sharepoint.com/personal/ibinfo_bcpsecurities_com/Documents/Documentos/Market Update Automation/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="37" documentId="8_{94004D96-580F-404F-B8DE-3B882EEF74BA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{5B9BC5A7-637A-4829-BD7C-911136EF458D}"/>
+  <xr:revisionPtr revIDLastSave="41" documentId="8_{94004D96-580F-404F-B8DE-3B882EEF74BA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{4FDB21CB-1208-46AA-BBFF-EB7C2173F4F2}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{E8956822-5CC2-4023-927E-A7F8B7EA2433}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="16" uniqueCount="16">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="24" uniqueCount="24">
   <si>
     <t>DK261868 Corp</t>
   </si>
@@ -80,13 +80,37 @@
     <t>DH675361 Corp</t>
   </si>
   <si>
-    <t>DH669881 Corp</t>
-  </si>
-  <si>
     <t>DH675309 Corp</t>
   </si>
   <si>
-    <t>DK239508 Corp</t>
+    <t>DQ529284 Corp</t>
+  </si>
+  <si>
+    <t>YI917676 Corp</t>
+  </si>
+  <si>
+    <t>DI473077 Corp</t>
+  </si>
+  <si>
+    <t>YI303525 Corp</t>
+  </si>
+  <si>
+    <t>DI473076 Corp</t>
+  </si>
+  <si>
+    <t>DI473078 Corp</t>
+  </si>
+  <si>
+    <t>DJ619870 Corp</t>
+  </si>
+  <si>
+    <t>DI842712 Corp</t>
+  </si>
+  <si>
+    <t>DC966977 Corp</t>
+  </si>
+  <si>
+    <t>DH155131 Corp</t>
   </si>
 </sst>
 </file>
@@ -151,7 +175,7 @@
       <tp t="e">
         <v>#N/A</v>
         <stp/>
-        <stp>BSRCH|9556213794820606431</stp>
+        <stp>BSRCH|11776511492595393546</stp>
         <tr r="A1" s="1"/>
       </tp>
     </main>
@@ -476,47 +500,48 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FDFCE30C-E6A3-4CE0-8A56-2BFB70ACD271}">
-  <dimension ref="A1:F17"/>
+  <dimension ref="A1:F25"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
+    <col min="1" max="1" width="13.85546875" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="22.140625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:6" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" t="str">
-        <f>_xll.BSRCH("FI:New Issues Brazil","cols=1;rows=17")</f>
+        <f>_xll.BSRCH("FI:New Issues Brazil - EB2","cols=1;rows=25")</f>
         <v>id</v>
       </c>
       <c r="F1" s="1"/>
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>0</v>
+        <v>14</v>
       </c>
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>1</v>
+        <v>15</v>
       </c>
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>2</v>
+        <v>4</v>
       </c>
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="6" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>4</v>
+        <v>0</v>
       </c>
     </row>
     <row r="7" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>5</v>
+        <v>3</v>
       </c>
     </row>
     <row r="8" spans="1:6" x14ac:dyDescent="0.25">
@@ -526,47 +551,87 @@
     </row>
     <row r="9" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>7</v>
+        <v>16</v>
       </c>
     </row>
     <row r="10" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>8</v>
+        <v>5</v>
       </c>
     </row>
     <row r="11" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>9</v>
+        <v>17</v>
       </c>
     </row>
     <row r="12" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>10</v>
+        <v>18</v>
       </c>
     </row>
     <row r="13" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>11</v>
+        <v>2</v>
       </c>
     </row>
     <row r="14" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>12</v>
+        <v>19</v>
       </c>
     </row>
     <row r="15" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>13</v>
+        <v>20</v>
       </c>
     </row>
     <row r="16" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
-        <v>14</v>
+        <v>21</v>
       </c>
     </row>
     <row r="17" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
-        <v>15</v>
+        <v>7</v>
+      </c>
+    </row>
+    <row r="18" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A18" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="19" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A19" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="20" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A20" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="21" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A21" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="22" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A22" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="23" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A23" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="24" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A24" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="25" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A25" t="s">
+        <v>23</v>
       </c>
     </row>
   </sheetData>

</xml_diff>